<commit_message>
Refactor: move structured data to Excel, clean up AGENT.md
</commit_message>
<xml_diff>
--- a/Job_Search_Tracker.xlsx
+++ b/Job_Search_Tracker.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -636,6 +636,86 @@
       <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Applied via LinkedIn Easy Apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Flipkart</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Android SDE</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Weekday AI</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Android Developer</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Snapmint</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Android Developer</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Innoventes Technologies</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Android Developer</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2519,6 +2599,106 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Flipkart</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Android SDE</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Weekday AI</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Android Developer</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Snapmint</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Android Developer</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Innoventes Technologies</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Android Developer</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Send referral messages to all 6 PhonePe contacts; update tracker
</commit_message>
<xml_diff>
--- a/Job_Search_Tracker.xlsx
+++ b/Job_Search_Tracker.xlsx
@@ -858,13 +858,17 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>not_sent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr"/>
@@ -916,13 +920,17 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>not_sent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr"/>
@@ -974,13 +982,17 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>not_sent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr"/>
@@ -1140,13 +1152,17 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>not_sent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr"/>
@@ -1360,13 +1376,17 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>not_sent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr"/>
@@ -1526,13 +1546,17 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>not_sent</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Send Couchbase referral messages to 4 accepted contacts; update tracker
</commit_message>
<xml_diff>
--- a/Job_Search_Tracker.xlsx
+++ b/Job_Search_Tracker.xlsx
@@ -2038,19 +2038,27 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
           <t>pending</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr"/>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="inlineStr"/>
-      <c r="K23" s="6" t="inlineStr">
-        <is>
-          <t>not_sent</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
@@ -2096,19 +2104,27 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
           <t>pending</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>not_sent</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr"/>
@@ -2208,19 +2224,27 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
           <t>pending</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>not_sent</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr"/>
@@ -2316,19 +2340,27 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
           <t>pending</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>not_sent</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr"/>

</xml_diff>